<commit_message>
Restore export commands and speed up reports
</commit_message>
<xml_diff>
--- a/templates/template_horeca.xlsx
+++ b/templates/template_horeca.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\KB_Market_Survey_Telegram_V33_14_KHMER_SUMMARY_RENDER_FIXED\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC197F73-11DC-41D4-968F-F5C3107EC778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7E0C80-537B-4976-A256-3A97BE95FE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
+  <si>
+    <t>Market Improvement Report</t>
+  </si>
   <si>
     <t>Dealer :                                                      Report Date:</t>
   </si>
@@ -64,9 +67,45 @@
     <t xml:space="preserve">Motor Shop: </t>
   </si>
   <si>
+    <t>New Outlet Purchase</t>
+  </si>
+  <si>
     <t>Volume</t>
   </si>
   <si>
+    <t>CAMBODIA COLA</t>
+  </si>
+  <si>
+    <t>WURKZ</t>
+  </si>
+  <si>
+    <t>DAZZ</t>
+  </si>
+  <si>
+    <t>DAZZ Zero Sugar</t>
+  </si>
+  <si>
+    <t>IZE PET 300ml Flavour</t>
+  </si>
+  <si>
+    <t>IZE COLA PET 1.5L All SKUs</t>
+  </si>
+  <si>
+    <t>Wurkz Ice</t>
+  </si>
+  <si>
+    <t>CAMBODIA Sport 300mL</t>
+  </si>
+  <si>
+    <t>CAMBODIA Sport 500mL</t>
+  </si>
+  <si>
+    <t>CAMBODIA WATER 500mL</t>
+  </si>
+  <si>
+    <t>CAMBODIA WATER 1500mL</t>
+  </si>
+  <si>
     <t>PRODUCT MOVEMENT VS COMPETITOR</t>
   </si>
   <si>
@@ -88,6 +127,102 @@
     <t>Ring Pull</t>
   </si>
   <si>
+    <t>CAMBODIA COLA 330ml</t>
+  </si>
+  <si>
+    <t>Coca Cola 330ml</t>
+  </si>
+  <si>
+    <t>Boostrong</t>
+  </si>
+  <si>
+    <t>Krud ED</t>
+  </si>
+  <si>
+    <t>Champion</t>
+  </si>
+  <si>
+    <t>King Kong</t>
+  </si>
+  <si>
+    <t>Krud Ice</t>
+  </si>
+  <si>
+    <t>Super Boostrong</t>
+  </si>
+  <si>
+    <t>AIRA</t>
+  </si>
+  <si>
+    <t>BACCHUSE</t>
+  </si>
+  <si>
+    <t>Dragon</t>
+  </si>
+  <si>
+    <t>BACCHUSE Sugar Free</t>
+  </si>
+  <si>
+    <t>IZE PET 300ml All SKUs</t>
+  </si>
+  <si>
+    <t>POP Z Flavour</t>
+  </si>
+  <si>
+    <t>Big Cola 3L</t>
+  </si>
+  <si>
+    <t>V Cola 350ml</t>
+  </si>
+  <si>
+    <t>Coca 1.5L</t>
+  </si>
+  <si>
+    <t>Sting Can 330ml</t>
+  </si>
+  <si>
+    <t>EXPREZ Can 330ml</t>
+  </si>
+  <si>
+    <t>Pocari Sweat</t>
+  </si>
+  <si>
+    <t>Idol Can 330ml</t>
+  </si>
+  <si>
+    <t>CAMBODIA Sport 500ml</t>
+  </si>
+  <si>
+    <t>CAMBODIA Sport 300ml</t>
+  </si>
+  <si>
+    <t>Provida 500mL</t>
+  </si>
+  <si>
+    <t>V-Active Sport</t>
+  </si>
+  <si>
+    <t>Vital 500mL</t>
+  </si>
+  <si>
+    <t>Provida 1500mL</t>
+  </si>
+  <si>
+    <t>Ganzberg  500ml</t>
+  </si>
+  <si>
+    <t>Hitech 500mL</t>
+  </si>
+  <si>
+    <t>Vital 1500mL</t>
+  </si>
+  <si>
+    <t>Ganzberg 1500ml</t>
+  </si>
+  <si>
+    <t>Hitech 1500mL</t>
+  </si>
+  <si>
     <t>Ring Pull In Outlets</t>
   </si>
   <si>
@@ -118,163 +253,58 @@
     <t>4.</t>
   </si>
   <si>
-    <t>CB Pint</t>
-  </si>
-  <si>
-    <t>CB SUPEEME Pint</t>
+    <t>CBC 4.4 NCP</t>
+  </si>
+  <si>
+    <t>CB Original NCP</t>
+  </si>
+  <si>
+    <t>CB LITE NCP</t>
+  </si>
+  <si>
+    <t>CB BLACK NCP</t>
+  </si>
+  <si>
+    <t>CAMBODIA ED</t>
+  </si>
+  <si>
+    <t>EXPREZ Melon</t>
   </si>
   <si>
     <t>CB LITE ORD</t>
   </si>
   <si>
-    <t>CBC 4.4 NCP</t>
-  </si>
-  <si>
-    <t>CB Original NCP</t>
-  </si>
-  <si>
-    <t>CB BLACK NCP</t>
-  </si>
-  <si>
-    <t>CAMBODIA COLA</t>
-  </si>
-  <si>
-    <t>WURKZ</t>
-  </si>
-  <si>
-    <t>CAMBODIA ED</t>
-  </si>
-  <si>
-    <t>DAZZ</t>
-  </si>
-  <si>
-    <t>DAZZ Zero Sugar</t>
-  </si>
-  <si>
-    <t>EXPREZ Can 330ml</t>
-  </si>
-  <si>
-    <t>CAMBODIA Sport 300mL</t>
-  </si>
-  <si>
-    <t>CAMBODIA Sport 500mL</t>
-  </si>
-  <si>
-    <t>CAMBODIA WATER 500mL</t>
-  </si>
-  <si>
-    <t>Tiger Pint</t>
-  </si>
-  <si>
-    <t>Angkor Pint</t>
-  </si>
-  <si>
     <t>GB SNOW ORD</t>
   </si>
   <si>
+    <t>GB SNOW NCP</t>
+  </si>
+  <si>
     <t>HANUMAN LITE ORD</t>
   </si>
   <si>
+    <t>GB Original NCP</t>
+  </si>
+  <si>
+    <t>Hanuman LITE NCP</t>
+  </si>
+  <si>
+    <t>Hanuman Black NCP</t>
+  </si>
+  <si>
+    <t>King Kong Ice</t>
+  </si>
+  <si>
     <t>Krud LITE ORD</t>
   </si>
   <si>
-    <t>GB Original NCP</t>
-  </si>
-  <si>
     <t>Krud NCP</t>
   </si>
   <si>
-    <t>GB SNOW NCP</t>
-  </si>
-  <si>
-    <t>Hanuman LITE NCP</t>
-  </si>
-  <si>
     <t>Krud LITE NCP</t>
   </si>
   <si>
     <t>Greet LITE NCP</t>
-  </si>
-  <si>
-    <t>Hanuman Black NCP</t>
-  </si>
-  <si>
-    <t>Coca Cola 330ml</t>
-  </si>
-  <si>
-    <t>Boostrong</t>
-  </si>
-  <si>
-    <t>Krud ED</t>
-  </si>
-  <si>
-    <t>BACCHUSE</t>
-  </si>
-  <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>BACCHUSE Sugar Free</t>
-  </si>
-  <si>
-    <t>Sting Can 330ml</t>
-  </si>
-  <si>
-    <t>Idol Can 330ml</t>
-  </si>
-  <si>
-    <t>Pocari Sweat</t>
-  </si>
-  <si>
-    <t>V-Active Sport</t>
-  </si>
-  <si>
-    <t>Vital 500mL</t>
-  </si>
-  <si>
-    <t>Provida 500mL</t>
-  </si>
-  <si>
-    <t>Ganzberg 500ml</t>
-  </si>
-  <si>
-    <t>Hitech 500mL</t>
-  </si>
-  <si>
-    <t>Market Improvement Report HORECA</t>
-  </si>
-  <si>
-    <t>CBL Pint</t>
-  </si>
-  <si>
-    <t>CB Black Pint</t>
-  </si>
-  <si>
-    <t>HANUMAN LITE Pint</t>
-  </si>
-  <si>
-    <t>Tiger Crystal Pint</t>
-  </si>
-  <si>
-    <t>Vathanac LITE Pint</t>
-  </si>
-  <si>
-    <t>ABC Pint</t>
-  </si>
-  <si>
-    <t>V Cola 330ml</t>
-  </si>
-  <si>
-    <t>EXPREZ Melon</t>
-  </si>
-  <si>
-    <t>Dragon Pint</t>
-  </si>
-  <si>
-    <t>HANUMAN Black Pint</t>
-  </si>
-  <si>
-    <t>Local Drink:</t>
   </si>
 </sst>
 </file>
@@ -338,7 +368,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -392,24 +422,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -443,48 +460,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -537,6 +545,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -545,7 +556,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -587,9 +598,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -602,12 +613,52 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525">
@@ -665,7 +716,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -691,7 +742,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -720,7 +771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA48"/>
+  <dimension ref="A1:AA49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -747,8 +798,8 @@
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
-        <v>73</v>
+      <c r="A2" s="25" t="s">
+        <v>0</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -778,8 +829,8 @@
       <c r="AA2" s="14"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
-        <v>0</v>
+      <c r="A3" s="13" t="s">
+        <v>1</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -809,19 +860,19 @@
       <c r="AA3" s="14"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="19" t="s">
-        <v>1</v>
+      <c r="A4" s="18" t="s">
+        <v>2</v>
       </c>
       <c r="B4" s="12"/>
-      <c r="C4" s="19" t="s">
-        <v>2</v>
+      <c r="C4" s="18" t="s">
+        <v>3</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="19" t="s">
-        <v>3</v>
+      <c r="H4" s="18" t="s">
+        <v>4</v>
       </c>
       <c r="I4" s="11"/>
       <c r="J4" s="11"/>
@@ -837,17 +888,17 @@
       <c r="T4" s="11"/>
       <c r="U4" s="11"/>
       <c r="V4" s="12"/>
-      <c r="W4" s="19" t="s">
-        <v>4</v>
+      <c r="W4" s="18" t="s">
+        <v>5</v>
       </c>
       <c r="X4" s="11"/>
       <c r="Y4" s="11"/>
       <c r="Z4" s="11"/>
       <c r="AA4" s="12"/>
     </row>
-    <row r="5" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="24" t="s">
-        <v>5</v>
+    <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="15" t="s">
+        <v>6</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -878,51 +929,51 @@
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="28" t="s">
         <v>8</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>9</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="20" t="s">
-        <v>9</v>
+      <c r="H6" s="16" t="s">
+        <v>10</v>
       </c>
       <c r="I6" s="11"/>
       <c r="J6" s="11"/>
       <c r="K6" s="12"/>
-      <c r="L6" s="20" t="s">
-        <v>10</v>
+      <c r="L6" s="16" t="s">
+        <v>11</v>
       </c>
       <c r="M6" s="11"/>
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
-      <c r="P6" s="20" t="s">
-        <v>11</v>
+      <c r="P6" s="16" t="s">
+        <v>12</v>
       </c>
       <c r="Q6" s="11"/>
       <c r="R6" s="11"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="20" t="s">
-        <v>12</v>
+      <c r="T6" s="16" t="s">
+        <v>13</v>
       </c>
       <c r="U6" s="11"/>
       <c r="V6" s="12"/>
-      <c r="W6" s="27" t="s">
-        <v>13</v>
+      <c r="W6" s="19" t="s">
+        <v>14</v>
       </c>
       <c r="X6" s="11"/>
       <c r="Y6" s="12"/>
       <c r="Z6" s="9" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -930,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="11"/>
@@ -958,12 +1009,12 @@
       <c r="Z7" s="3"/>
       <c r="AA7" s="3"/>
     </row>
-    <row r="8" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="11"/>
@@ -991,12 +1042,12 @@
       <c r="Z8" s="3"/>
       <c r="AA8" s="3"/>
     </row>
-    <row r="9" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="11"/>
@@ -1024,12 +1075,12 @@
       <c r="Z9" s="3"/>
       <c r="AA9" s="3"/>
     </row>
-    <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="11"/>
@@ -1062,31 +1113,31 @@
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
-      <c r="S11" s="17"/>
-      <c r="T11" s="15"/>
-      <c r="U11" s="16"/>
-      <c r="V11" s="17"/>
-      <c r="W11" s="15"/>
-      <c r="X11" s="16"/>
-      <c r="Y11" s="17"/>
+        <v>80</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="12"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="12"/>
       <c r="Z11" s="3"/>
       <c r="AA11" s="3"/>
     </row>
@@ -1095,7 +1146,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
@@ -1128,7 +1179,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
@@ -1161,7 +1212,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
@@ -1194,7 +1245,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
@@ -1227,7 +1278,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
@@ -1260,7 +1311,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
@@ -1293,7 +1344,7 @@
         <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
@@ -1321,12 +1372,12 @@
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
     </row>
-    <row r="19" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
@@ -1354,22 +1405,22 @@
       <c r="Z19" s="3"/>
       <c r="AA19" s="3"/>
     </row>
-    <row r="20" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>14</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
       <c r="G20" s="12"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="17"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="12"/>
       <c r="L20" s="10"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -1387,12 +1438,12 @@
       <c r="Z20" s="3"/>
       <c r="AA20" s="3"/>
     </row>
-    <row r="21" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
@@ -1420,12 +1471,12 @@
       <c r="Z21" s="3"/>
       <c r="AA21" s="3"/>
     </row>
-    <row r="22" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>16</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
@@ -1453,12 +1504,12 @@
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
     </row>
-    <row r="23" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
@@ -1486,12 +1537,12 @@
       <c r="Z23" s="3"/>
       <c r="AA23" s="3"/>
     </row>
-    <row r="24" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
@@ -1519,9 +1570,9 @@
       <c r="Z24" s="3"/>
       <c r="AA24" s="3"/>
     </row>
-    <row r="25" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="18" t="s">
-        <v>15</v>
+    <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>28</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -1550,95 +1601,95 @@
       <c r="Z25" s="14"/>
       <c r="AA25" s="14"/>
     </row>
-    <row r="26" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="Q26" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="R26" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="T26" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="U26" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="V26" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="W26" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X26" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="Y26" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="Z26" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="AA26" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="3">
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1646,20 +1697,22 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="1" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="1" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
-      <c r="R27" s="1"/>
+      <c r="R27" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
@@ -1670,12 +1723,12 @@
       <c r="Z27" s="3"/>
       <c r="AA27" s="3"/>
     </row>
-    <row r="28" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
         <v>2</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1683,29 +1736,27 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="1" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
       <c r="R28" s="1" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
-      <c r="W28" s="1" t="s">
-        <v>78</v>
-      </c>
+      <c r="W28" s="1"/>
       <c r="X28" s="3"/>
       <c r="Y28" s="3"/>
       <c r="Z28" s="3"/>
@@ -1716,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1724,27 +1775,29 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
-      <c r="W29" s="1"/>
+      <c r="W29" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
@@ -1755,30 +1808,26 @@
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="H30" s="1"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="1" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
-      <c r="R30" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="R30" s="1"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
@@ -1802,15 +1851,13 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
-      <c r="M31" s="1" t="s">
-        <v>53</v>
-      </c>
+      <c r="M31" s="1"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -1831,7 +1878,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -1839,29 +1886,25 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
-      <c r="M32" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="M32" s="1"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
       <c r="R32" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
-      <c r="W32" s="1" t="s">
-        <v>57</v>
-      </c>
+      <c r="W32" s="1"/>
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
       <c r="Z32" s="3"/>
@@ -1872,7 +1915,7 @@
         <v>7</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -1880,18 +1923,22 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="1" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
-      <c r="M33" s="1"/>
+      <c r="M33" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
-      <c r="R33" s="1"/>
+      <c r="R33" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
@@ -1907,7 +1954,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -1915,20 +1962,22 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="1" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="1" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
-      <c r="R34" s="1"/>
+      <c r="R34" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
@@ -1944,7 +1993,7 @@
         <v>9</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1952,7 +2001,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
@@ -1964,7 +2013,7 @@
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="1" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
@@ -1981,14 +2030,16 @@
         <v>10</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="1"/>
+      <c r="H36" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
@@ -2014,7 +2065,7 @@
         <v>11</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -2022,7 +2073,7 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="1" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
@@ -2034,7 +2085,7 @@
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
       <c r="R37" s="1" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
@@ -2051,7 +2102,7 @@
         <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -2059,13 +2110,15 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="1" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
-      <c r="M38" s="1"/>
+      <c r="M38" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
@@ -2086,7 +2139,7 @@
         <v>13</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -2094,21 +2147,21 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="1" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
       <c r="R39" s="1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
@@ -2125,7 +2178,7 @@
         <v>14</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -2133,21 +2186,21 @@
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="1" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="1" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
       <c r="R40" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
@@ -2164,7 +2217,7 @@
         <v>15</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -2172,28 +2225,28 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="1" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
       <c r="R41" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
       <c r="W41" s="1" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
@@ -2201,66 +2254,72 @@
       <c r="AA41" s="3"/>
     </row>
     <row r="42" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
+      <c r="A42" s="3">
+        <v>16</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+      <c r="P42" s="3"/>
+      <c r="Q42" s="3"/>
+      <c r="R42" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
+      <c r="U42" s="3"/>
+      <c r="V42" s="3"/>
+      <c r="W42" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="X42" s="3"/>
+      <c r="Y42" s="3"/>
+      <c r="Z42" s="3"/>
+      <c r="AA42" s="3"/>
     </row>
     <row r="43" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B43" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43" s="12"/>
-      <c r="D43" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="G43" s="12"/>
-      <c r="I43" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="14"/>
-      <c r="M43" s="14"/>
-      <c r="N43" s="14"/>
-      <c r="O43" s="14"/>
-      <c r="P43" s="14"/>
-      <c r="Q43" s="14"/>
-      <c r="S43" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="T43" s="14"/>
-      <c r="U43" s="14"/>
-      <c r="V43" s="14"/>
-      <c r="W43" s="14"/>
-      <c r="X43" s="14"/>
-      <c r="Y43" s="14"/>
-      <c r="Z43" s="14"/>
-      <c r="AA43" s="14"/>
-    </row>
-    <row r="44" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="3">
-        <v>1</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>27</v>
+      <c r="A43" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+    </row>
+    <row r="44" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B44" s="23" t="s">
+        <v>8</v>
       </c>
       <c r="C44" s="12"/>
-      <c r="D44" s="10"/>
+      <c r="D44" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="E44" s="12"/>
-      <c r="F44" s="10"/>
+      <c r="F44" s="24" t="s">
+        <v>69</v>
+      </c>
       <c r="G44" s="12"/>
-      <c r="I44" s="18">
-        <v>1</v>
+      <c r="I44" s="22" t="s">
+        <v>70</v>
       </c>
       <c r="J44" s="14"/>
       <c r="K44" s="14"/>
@@ -2270,8 +2329,8 @@
       <c r="O44" s="14"/>
       <c r="P44" s="14"/>
       <c r="Q44" s="14"/>
-      <c r="S44" s="18">
-        <v>1</v>
+      <c r="S44" s="22" t="s">
+        <v>71</v>
       </c>
       <c r="T44" s="14"/>
       <c r="U44" s="14"/>
@@ -2282,20 +2341,20 @@
       <c r="Z44" s="14"/>
       <c r="AA44" s="14"/>
     </row>
-    <row r="45" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
-        <v>2</v>
-      </c>
-      <c r="B45" s="24" t="s">
-        <v>28</v>
+        <v>1</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="10"/>
       <c r="E45" s="12"/>
       <c r="F45" s="10"/>
       <c r="G45" s="12"/>
-      <c r="I45" s="18" t="s">
-        <v>29</v>
+      <c r="I45" s="13">
+        <v>1</v>
       </c>
       <c r="J45" s="14"/>
       <c r="K45" s="14"/>
@@ -2305,8 +2364,8 @@
       <c r="O45" s="14"/>
       <c r="P45" s="14"/>
       <c r="Q45" s="14"/>
-      <c r="S45" s="18">
-        <v>2</v>
+      <c r="S45" s="13">
+        <v>1</v>
       </c>
       <c r="T45" s="14"/>
       <c r="U45" s="14"/>
@@ -2317,16 +2376,20 @@
       <c r="Z45" s="14"/>
       <c r="AA45" s="14"/>
     </row>
-    <row r="46" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="5"/>
-      <c r="B46" s="21"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="14"/>
-      <c r="I46" s="18" t="s">
-        <v>30</v>
+    <row r="46" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="3">
+        <v>2</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" s="12"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="12"/>
+      <c r="I46" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="J46" s="14"/>
       <c r="K46" s="14"/>
@@ -2336,8 +2399,8 @@
       <c r="O46" s="14"/>
       <c r="P46" s="14"/>
       <c r="Q46" s="14"/>
-      <c r="S46" s="18">
-        <v>3</v>
+      <c r="S46" s="13">
+        <v>2</v>
       </c>
       <c r="T46" s="14"/>
       <c r="U46" s="14"/>
@@ -2348,16 +2411,16 @@
       <c r="Z46" s="14"/>
       <c r="AA46" s="14"/>
     </row>
-    <row r="47" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
-      <c r="B47" s="21"/>
+      <c r="B47" s="20"/>
       <c r="C47" s="14"/>
-      <c r="D47" s="21"/>
+      <c r="D47" s="20"/>
       <c r="E47" s="14"/>
-      <c r="F47" s="21"/>
+      <c r="F47" s="20"/>
       <c r="G47" s="14"/>
-      <c r="I47" s="18" t="s">
-        <v>31</v>
+      <c r="I47" s="13" t="s">
+        <v>75</v>
       </c>
       <c r="J47" s="14"/>
       <c r="K47" s="14"/>
@@ -2367,8 +2430,8 @@
       <c r="O47" s="14"/>
       <c r="P47" s="14"/>
       <c r="Q47" s="14"/>
-      <c r="S47" s="18" t="s">
-        <v>31</v>
+      <c r="S47" s="13">
+        <v>3</v>
       </c>
       <c r="T47" s="14"/>
       <c r="U47" s="14"/>
@@ -2379,157 +2442,188 @@
       <c r="Z47" s="14"/>
       <c r="AA47" s="14"/>
     </row>
-    <row r="48" spans="1:27" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="5"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="14"/>
+      <c r="I48" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
+      <c r="L48" s="14"/>
+      <c r="M48" s="14"/>
+      <c r="N48" s="14"/>
+      <c r="O48" s="14"/>
+      <c r="P48" s="14"/>
+      <c r="Q48" s="14"/>
+      <c r="S48" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="T48" s="14"/>
+      <c r="U48" s="14"/>
+      <c r="V48" s="14"/>
+      <c r="W48" s="14"/>
+      <c r="X48" s="14"/>
+      <c r="Y48" s="14"/>
+      <c r="Z48" s="14"/>
+      <c r="AA48" s="14"/>
+    </row>
+    <row r="49" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="148">
+    <mergeCell ref="I44:Q44"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="P21:S21"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="S48:AA48"/>
+    <mergeCell ref="H4:V4"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="I45:Q45"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="W8:Y8"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="T20:V20"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="I48:Q48"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="T24:V24"/>
+    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="S45:AA45"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="P20:S20"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="T12:V12"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="S44:AA44"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="S47:AA47"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="A5:AA5"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="W20:Y20"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="S46:AA46"/>
+    <mergeCell ref="P22:S22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="P9:S9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="P24:S24"/>
+    <mergeCell ref="A25:AA25"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:V7"/>
+    <mergeCell ref="W7:Y7"/>
     <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="H21:K21"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="W6:Y6"/>
     <mergeCell ref="C6:G6"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="T10:V10"/>
     <mergeCell ref="P8:S8"/>
     <mergeCell ref="H8:K8"/>
     <mergeCell ref="W4:AA4"/>
     <mergeCell ref="L6:O6"/>
-    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="T13:V13"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A25:AA25"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="W20:Y20"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:V7"/>
-    <mergeCell ref="W7:Y7"/>
-    <mergeCell ref="A5:AA5"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="P24:S24"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="P9:S9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="T13:V13"/>
-    <mergeCell ref="P18:S18"/>
-    <mergeCell ref="W12:Y12"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="P15:S15"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="S44:AA44"/>
-    <mergeCell ref="W17:Y17"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="P21:S21"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="S43:AA43"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="I43:Q43"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="W19:Y19"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="P20:S20"/>
-    <mergeCell ref="T20:V20"/>
-    <mergeCell ref="S47:AA47"/>
-    <mergeCell ref="H4:V4"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="I44:Q44"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="I45:Q45"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="P22:S22"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="T12:V12"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="W18:Y18"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="L10:O10"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="C20:G20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Prevent legacy Ring Pull block in GT HORECA reports
</commit_message>
<xml_diff>
--- a/templates/template_horeca.xlsx
+++ b/templates/template_horeca.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\KB_Market_Survey_Telegram_V33_14_KHMER_SUMMARY_RENDER_FIXED\backend\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7E0C80-537B-4976-A256-3A97BE95FE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE25A39B-599A-48A9-9AFB-8CA7DC4443E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="91">
   <si>
     <t>Market Improvement Report</t>
   </si>
@@ -223,27 +223,12 @@
     <t>Hitech 1500mL</t>
   </si>
   <si>
-    <t>Ring Pull In Outlets</t>
-  </si>
-  <si>
-    <t>Total Outlets</t>
-  </si>
-  <si>
-    <t>Ring Pull Qty (Can)</t>
-  </si>
-  <si>
     <t>Key Issues</t>
   </si>
   <si>
     <t>INITIATIVE IDEA / SUGGESTION</t>
   </si>
   <si>
-    <t>CBL NCP 6 Can</t>
-  </si>
-  <si>
-    <t>CBL NCP 5 USD</t>
-  </si>
-  <si>
     <t>2.</t>
   </si>
   <si>
@@ -305,13 +290,16 @@
   </si>
   <si>
     <t>Greet LITE NCP</t>
+  </si>
+  <si>
+    <t>ចំណុចដួល</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,6 +336,11 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="17"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans Khmer"/>
     </font>
   </fonts>
   <fills count="4">
@@ -440,9 +433,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -455,45 +445,44 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -771,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA49"/>
+  <dimension ref="A1:AA47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -794,138 +783,138 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="68" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6"/>
-      <c r="D1" s="7"/>
+      <c r="A1" s="5"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-      <c r="W3" s="14"/>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14"/>
-      <c r="Z3" s="14"/>
-      <c r="AA3" s="14"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="18" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="18" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="12"/>
-      <c r="W4" s="18" t="s">
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="13"/>
+      <c r="W4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="X4" s="11"/>
-      <c r="Y4" s="11"/>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="13"/>
     </row>
     <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11"/>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="11"/>
-      <c r="AA5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="13"/>
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
@@ -934,45 +923,45 @@
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="13"/>
       <c r="H6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="13"/>
       <c r="L6" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="13"/>
       <c r="P6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="13"/>
       <c r="T6" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="U6" s="11"/>
-      <c r="V6" s="12"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="13"/>
       <c r="W6" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="X6" s="11"/>
-      <c r="Y6" s="12"/>
-      <c r="Z6" s="9" t="s">
+      <c r="X6" s="12"/>
+      <c r="Y6" s="13"/>
+      <c r="Z6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="AA6" s="8" t="s">
+      <c r="AA6" s="7" t="s">
         <v>16</v>
       </c>
     </row>
@@ -981,31 +970,31 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="12"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="12"/>
-      <c r="W7" s="10"/>
-      <c r="X7" s="11"/>
-      <c r="Y7" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="13"/>
+      <c r="T7" s="11"/>
+      <c r="U7" s="12"/>
+      <c r="V7" s="13"/>
+      <c r="W7" s="11"/>
+      <c r="X7" s="12"/>
+      <c r="Y7" s="13"/>
       <c r="Z7" s="3"/>
       <c r="AA7" s="3"/>
     </row>
@@ -1014,31 +1003,31 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="12"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="12"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="11"/>
-      <c r="Y8" s="12"/>
+        <v>72</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="13"/>
+      <c r="T8" s="11"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="13"/>
+      <c r="W8" s="11"/>
+      <c r="X8" s="12"/>
+      <c r="Y8" s="13"/>
       <c r="Z8" s="3"/>
       <c r="AA8" s="3"/>
     </row>
@@ -1047,31 +1036,31 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="11"/>
-      <c r="S9" s="12"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="11"/>
-      <c r="V9" s="12"/>
-      <c r="W9" s="10"/>
-      <c r="X9" s="11"/>
-      <c r="Y9" s="12"/>
+        <v>73</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="13"/>
+      <c r="T9" s="11"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="13"/>
+      <c r="W9" s="11"/>
+      <c r="X9" s="12"/>
+      <c r="Y9" s="13"/>
       <c r="Z9" s="3"/>
       <c r="AA9" s="3"/>
     </row>
@@ -1080,31 +1069,31 @@
         <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="11"/>
-      <c r="V10" s="12"/>
-      <c r="W10" s="10"/>
-      <c r="X10" s="11"/>
-      <c r="Y10" s="12"/>
+        <v>74</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="11"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="11"/>
+      <c r="X10" s="12"/>
+      <c r="Y10" s="13"/>
       <c r="Z10" s="3"/>
       <c r="AA10" s="3"/>
     </row>
@@ -1113,31 +1102,31 @@
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
-      <c r="S11" s="12"/>
-      <c r="T11" s="10"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="12"/>
-      <c r="W11" s="10"/>
-      <c r="X11" s="11"/>
-      <c r="Y11" s="12"/>
+        <v>75</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="13"/>
+      <c r="T11" s="11"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="13"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="12"/>
+      <c r="Y11" s="13"/>
       <c r="Z11" s="3"/>
       <c r="AA11" s="3"/>
     </row>
@@ -1148,29 +1137,29 @@
       <c r="B12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="12"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="12"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="11"/>
-      <c r="Y12" s="12"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="13"/>
+      <c r="T12" s="11"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="13"/>
+      <c r="W12" s="11"/>
+      <c r="X12" s="12"/>
+      <c r="Y12" s="13"/>
       <c r="Z12" s="3"/>
       <c r="AA12" s="3"/>
     </row>
@@ -1181,29 +1170,29 @@
       <c r="B13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="12"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="12"/>
-      <c r="W13" s="10"/>
-      <c r="X13" s="11"/>
-      <c r="Y13" s="12"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="13"/>
+      <c r="T13" s="11"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="13"/>
+      <c r="W13" s="11"/>
+      <c r="X13" s="12"/>
+      <c r="Y13" s="13"/>
       <c r="Z13" s="3"/>
       <c r="AA13" s="3"/>
     </row>
@@ -1212,31 +1201,31 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="11"/>
-      <c r="S14" s="12"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="12"/>
-      <c r="W14" s="10"/>
-      <c r="X14" s="11"/>
-      <c r="Y14" s="12"/>
+        <v>76</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="13"/>
+      <c r="T14" s="11"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="13"/>
+      <c r="W14" s="11"/>
+      <c r="X14" s="12"/>
+      <c r="Y14" s="13"/>
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
     </row>
@@ -1247,29 +1236,29 @@
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
-      <c r="S15" s="12"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="12"/>
-      <c r="W15" s="10"/>
-      <c r="X15" s="11"/>
-      <c r="Y15" s="12"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="13"/>
+      <c r="T15" s="11"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="13"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="12"/>
+      <c r="Y15" s="13"/>
       <c r="Z15" s="3"/>
       <c r="AA15" s="3"/>
     </row>
@@ -1280,29 +1269,29 @@
       <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="12"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
-      <c r="S16" s="12"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="11"/>
-      <c r="V16" s="12"/>
-      <c r="W16" s="10"/>
-      <c r="X16" s="11"/>
-      <c r="Y16" s="12"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="13"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="13"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="12"/>
+      <c r="V16" s="13"/>
+      <c r="W16" s="11"/>
+      <c r="X16" s="12"/>
+      <c r="Y16" s="13"/>
       <c r="Z16" s="3"/>
       <c r="AA16" s="3"/>
     </row>
@@ -1313,29 +1302,29 @@
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="10"/>
-      <c r="U17" s="11"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="10"/>
-      <c r="X17" s="11"/>
-      <c r="Y17" s="12"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="13"/>
+      <c r="T17" s="11"/>
+      <c r="U17" s="12"/>
+      <c r="V17" s="13"/>
+      <c r="W17" s="11"/>
+      <c r="X17" s="12"/>
+      <c r="Y17" s="13"/>
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
     </row>
@@ -1346,29 +1335,29 @@
       <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="11"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="10"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="11"/>
-      <c r="Y18" s="12"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="11"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="13"/>
+      <c r="W18" s="11"/>
+      <c r="X18" s="12"/>
+      <c r="Y18" s="13"/>
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
     </row>
@@ -1377,31 +1366,31 @@
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="12"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="11"/>
-      <c r="Y19" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="13"/>
+      <c r="P19" s="11"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="11"/>
+      <c r="U19" s="12"/>
+      <c r="V19" s="13"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="12"/>
+      <c r="Y19" s="13"/>
       <c r="Z19" s="3"/>
       <c r="AA19" s="3"/>
     </row>
@@ -1412,29 +1401,29 @@
       <c r="B20" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="11"/>
-      <c r="V20" s="12"/>
-      <c r="W20" s="10"/>
-      <c r="X20" s="11"/>
-      <c r="Y20" s="12"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="13"/>
+      <c r="T20" s="11"/>
+      <c r="U20" s="12"/>
+      <c r="V20" s="13"/>
+      <c r="W20" s="11"/>
+      <c r="X20" s="12"/>
+      <c r="Y20" s="13"/>
       <c r="Z20" s="3"/>
       <c r="AA20" s="3"/>
     </row>
@@ -1445,29 +1434,29 @@
       <c r="B21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="12"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="12"/>
-      <c r="T21" s="10"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="12"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="11"/>
-      <c r="Y21" s="12"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="11"/>
+      <c r="U21" s="12"/>
+      <c r="V21" s="13"/>
+      <c r="W21" s="11"/>
+      <c r="X21" s="12"/>
+      <c r="Y21" s="13"/>
       <c r="Z21" s="3"/>
       <c r="AA21" s="3"/>
     </row>
@@ -1478,29 +1467,29 @@
       <c r="B22" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="12"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="12"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="12"/>
-      <c r="W22" s="10"/>
-      <c r="X22" s="11"/>
-      <c r="Y22" s="12"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="11"/>
+      <c r="U22" s="12"/>
+      <c r="V22" s="13"/>
+      <c r="W22" s="11"/>
+      <c r="X22" s="12"/>
+      <c r="Y22" s="13"/>
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
     </row>
@@ -1511,29 +1500,29 @@
       <c r="B23" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="12"/>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="11"/>
-      <c r="S23" s="12"/>
-      <c r="T23" s="10"/>
-      <c r="U23" s="11"/>
-      <c r="V23" s="12"/>
-      <c r="W23" s="10"/>
-      <c r="X23" s="11"/>
-      <c r="Y23" s="12"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="11"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="13"/>
+      <c r="T23" s="11"/>
+      <c r="U23" s="12"/>
+      <c r="V23" s="13"/>
+      <c r="W23" s="11"/>
+      <c r="X23" s="12"/>
+      <c r="Y23" s="13"/>
       <c r="Z23" s="3"/>
       <c r="AA23" s="3"/>
     </row>
@@ -1544,62 +1533,62 @@
       <c r="B24" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="12"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="12"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="12"/>
-      <c r="T24" s="10"/>
-      <c r="U24" s="11"/>
-      <c r="V24" s="12"/>
-      <c r="W24" s="10"/>
-      <c r="X24" s="11"/>
-      <c r="Y24" s="12"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="13"/>
+      <c r="T24" s="11"/>
+      <c r="U24" s="12"/>
+      <c r="V24" s="13"/>
+      <c r="W24" s="11"/>
+      <c r="X24" s="12"/>
+      <c r="Y24" s="13"/>
       <c r="Z24" s="3"/>
       <c r="AA24" s="3"/>
     </row>
     <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
-      <c r="R25" s="14"/>
-      <c r="S25" s="14"/>
-      <c r="T25" s="14"/>
-      <c r="U25" s="14"/>
-      <c r="V25" s="14"/>
-      <c r="W25" s="14"/>
-      <c r="X25" s="14"/>
-      <c r="Y25" s="14"/>
-      <c r="Z25" s="14"/>
-      <c r="AA25" s="14"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10"/>
+      <c r="W25" s="10"/>
+      <c r="X25" s="10"/>
+      <c r="Y25" s="10"/>
+      <c r="Z25" s="10"/>
+      <c r="AA25" s="10"/>
     </row>
     <row r="26" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
@@ -1689,7 +1678,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1697,21 +1686,21 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
       <c r="R27" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
@@ -1728,7 +1717,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1736,21 +1725,21 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="1" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
       <c r="R28" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -1767,7 +1756,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1775,28 +1764,28 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
@@ -1808,7 +1797,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1821,7 +1810,7 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
@@ -1930,7 +1919,7 @@
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
@@ -1954,7 +1943,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -2139,7 +2128,7 @@
         <v>13</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -2253,7 +2242,7 @@
       <c r="Z41" s="3"/>
       <c r="AA41" s="3"/>
     </row>
-    <row r="42" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3">
         <v>16</v>
       </c>
@@ -2294,318 +2283,188 @@
       <c r="Z42" s="3"/>
       <c r="AA42" s="3"/>
     </row>
-    <row r="43" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="13" t="s">
+    <row r="43" spans="1:27" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-    </row>
-    <row r="44" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B44" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="C44" s="12"/>
-      <c r="D44" s="17" t="s">
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
+      <c r="P43" s="22"/>
+      <c r="Q43" s="22"/>
+      <c r="R43" s="23"/>
+      <c r="S43" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E44" s="12"/>
-      <c r="F44" s="24" t="s">
+      <c r="T43" s="24"/>
+      <c r="U43" s="24"/>
+      <c r="V43" s="24"/>
+      <c r="W43" s="24"/>
+      <c r="X43" s="24"/>
+      <c r="Y43" s="24"/>
+      <c r="Z43" s="24"/>
+      <c r="AA43" s="24"/>
+    </row>
+    <row r="44" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="15">
+        <v>1</v>
+      </c>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="25">
+        <v>1</v>
+      </c>
+      <c r="J44" s="25"/>
+      <c r="K44" s="25"/>
+      <c r="L44" s="25"/>
+      <c r="M44" s="25"/>
+      <c r="N44" s="25"/>
+      <c r="O44" s="25"/>
+      <c r="P44" s="25"/>
+      <c r="Q44" s="25"/>
+      <c r="R44" s="23"/>
+      <c r="S44" s="25">
+        <v>1</v>
+      </c>
+      <c r="T44" s="24"/>
+      <c r="U44" s="24"/>
+      <c r="V44" s="24"/>
+      <c r="W44" s="24"/>
+      <c r="X44" s="24"/>
+      <c r="Y44" s="24"/>
+      <c r="Z44" s="24"/>
+      <c r="AA44" s="24"/>
+    </row>
+    <row r="45" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="15">
+        <v>2</v>
+      </c>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="G44" s="12"/>
-      <c r="I44" s="22" t="s">
+      <c r="J45" s="25"/>
+      <c r="K45" s="25"/>
+      <c r="L45" s="25"/>
+      <c r="M45" s="25"/>
+      <c r="N45" s="25"/>
+      <c r="O45" s="25"/>
+      <c r="P45" s="25"/>
+      <c r="Q45" s="25"/>
+      <c r="R45" s="23"/>
+      <c r="S45" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="T45" s="24"/>
+      <c r="U45" s="24"/>
+      <c r="V45" s="24"/>
+      <c r="W45" s="24"/>
+      <c r="X45" s="24"/>
+      <c r="Y45" s="24"/>
+      <c r="Z45" s="24"/>
+      <c r="AA45" s="24"/>
+    </row>
+    <row r="46" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="15">
+        <v>3</v>
+      </c>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="14"/>
-      <c r="M44" s="14"/>
-      <c r="N44" s="14"/>
-      <c r="O44" s="14"/>
-      <c r="P44" s="14"/>
-      <c r="Q44" s="14"/>
-      <c r="S44" s="22" t="s">
+      <c r="J46" s="25"/>
+      <c r="K46" s="25"/>
+      <c r="L46" s="25"/>
+      <c r="M46" s="25"/>
+      <c r="N46" s="25"/>
+      <c r="O46" s="25"/>
+      <c r="P46" s="25"/>
+      <c r="Q46" s="25"/>
+      <c r="R46" s="23"/>
+      <c r="S46" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="T46" s="24"/>
+      <c r="U46" s="24"/>
+      <c r="V46" s="24"/>
+      <c r="W46" s="24"/>
+      <c r="X46" s="24"/>
+      <c r="Y46" s="24"/>
+      <c r="Z46" s="24"/>
+      <c r="AA46" s="24"/>
+    </row>
+    <row r="47" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="15">
+        <v>4</v>
+      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="T44" s="14"/>
-      <c r="U44" s="14"/>
-      <c r="V44" s="14"/>
-      <c r="W44" s="14"/>
-      <c r="X44" s="14"/>
-      <c r="Y44" s="14"/>
-      <c r="Z44" s="14"/>
-      <c r="AA44" s="14"/>
-    </row>
-    <row r="45" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="3">
-        <v>1</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="C45" s="12"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="12"/>
-      <c r="I45" s="13">
-        <v>1</v>
-      </c>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-      <c r="L45" s="14"/>
-      <c r="M45" s="14"/>
-      <c r="N45" s="14"/>
-      <c r="O45" s="14"/>
-      <c r="P45" s="14"/>
-      <c r="Q45" s="14"/>
-      <c r="S45" s="13">
-        <v>1</v>
-      </c>
-      <c r="T45" s="14"/>
-      <c r="U45" s="14"/>
-      <c r="V45" s="14"/>
-      <c r="W45" s="14"/>
-      <c r="X45" s="14"/>
-      <c r="Y45" s="14"/>
-      <c r="Z45" s="14"/>
-      <c r="AA45" s="14"/>
-    </row>
-    <row r="46" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="3">
-        <v>2</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C46" s="12"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="12"/>
-      <c r="I46" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-      <c r="N46" s="14"/>
-      <c r="O46" s="14"/>
-      <c r="P46" s="14"/>
-      <c r="Q46" s="14"/>
-      <c r="S46" s="13">
-        <v>2</v>
-      </c>
-      <c r="T46" s="14"/>
-      <c r="U46" s="14"/>
-      <c r="V46" s="14"/>
-      <c r="W46" s="14"/>
-      <c r="X46" s="14"/>
-      <c r="Y46" s="14"/>
-      <c r="Z46" s="14"/>
-      <c r="AA46" s="14"/>
-    </row>
-    <row r="47" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="5"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="14"/>
-      <c r="I47" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="J47" s="14"/>
-      <c r="K47" s="14"/>
-      <c r="L47" s="14"/>
-      <c r="M47" s="14"/>
-      <c r="N47" s="14"/>
-      <c r="O47" s="14"/>
-      <c r="P47" s="14"/>
-      <c r="Q47" s="14"/>
-      <c r="S47" s="13">
-        <v>3</v>
-      </c>
-      <c r="T47" s="14"/>
-      <c r="U47" s="14"/>
-      <c r="V47" s="14"/>
-      <c r="W47" s="14"/>
-      <c r="X47" s="14"/>
-      <c r="Y47" s="14"/>
-      <c r="Z47" s="14"/>
-      <c r="AA47" s="14"/>
-    </row>
-    <row r="48" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="5"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="14"/>
-      <c r="I48" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
-      <c r="O48" s="14"/>
-      <c r="P48" s="14"/>
-      <c r="Q48" s="14"/>
-      <c r="S48" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="T48" s="14"/>
-      <c r="U48" s="14"/>
-      <c r="V48" s="14"/>
-      <c r="W48" s="14"/>
-      <c r="X48" s="14"/>
-      <c r="Y48" s="14"/>
-      <c r="Z48" s="14"/>
-      <c r="AA48" s="14"/>
-    </row>
-    <row r="49" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="J47" s="25"/>
+      <c r="K47" s="25"/>
+      <c r="L47" s="25"/>
+      <c r="M47" s="25"/>
+      <c r="N47" s="25"/>
+      <c r="O47" s="25"/>
+      <c r="P47" s="25"/>
+      <c r="Q47" s="25"/>
+      <c r="R47" s="23"/>
+      <c r="S47" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="T47" s="24"/>
+      <c r="U47" s="24"/>
+      <c r="V47" s="24"/>
+      <c r="W47" s="24"/>
+      <c r="X47" s="24"/>
+      <c r="Y47" s="24"/>
+      <c r="Z47" s="24"/>
+      <c r="AA47" s="24"/>
+    </row>
   </sheetData>
-  <mergeCells count="148">
-    <mergeCell ref="I44:Q44"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="W19:Y19"/>
-    <mergeCell ref="P21:S21"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="S48:AA48"/>
-    <mergeCell ref="H4:V4"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="I45:Q45"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="T20:V20"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="I48:Q48"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="T14:V14"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="W17:Y17"/>
+  <mergeCells count="136">
+    <mergeCell ref="A45:G45"/>
     <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="P18:S18"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="P20:S20"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="T12:V12"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="S44:AA44"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="S47:AA47"/>
-    <mergeCell ref="W18:Y18"/>
-    <mergeCell ref="A5:AA5"/>
-    <mergeCell ref="W12:Y12"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="W20:Y20"/>
-    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A46:G46"/>
     <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="P22:S22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="P9:S9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="P24:S24"/>
-    <mergeCell ref="A25:AA25"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="L7:O7"/>
     <mergeCell ref="P7:S7"/>
     <mergeCell ref="T7:V7"/>
@@ -2624,6 +2483,119 @@
     <mergeCell ref="L6:O6"/>
     <mergeCell ref="T13:V13"/>
     <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A5:AA5"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="W20:Y20"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="P22:S22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="P9:S9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="P24:S24"/>
+    <mergeCell ref="A25:AA25"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="P20:S20"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="S44:AA44"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="S47:AA47"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="S43:AA43"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="T12:V12"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="T20:V20"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="T24:V24"/>
+    <mergeCell ref="H4:V4"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="I45:Q45"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="W8:Y8"/>
+    <mergeCell ref="I44:Q44"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="P21:S21"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="C13:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>